<commit_message>
Add: new composition tests
</commit_message>
<xml_diff>
--- a/files/test_files/composicao_teste.xlsx
+++ b/files/test_files/composicao_teste.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Downloads\Projetos\filtercomp\files\test_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6BA0FEA-BA5F-425A-89EA-3B8F4E881A82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F94831D6-3B80-4C69-96A8-72CFBD965127}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2340" yWindow="2340" windowWidth="21600" windowHeight="11385" xr2:uid="{B01F5496-B8EA-4B4D-906B-0DA441535964}"/>
+    <workbookView xWindow="3120" yWindow="0" windowWidth="19485" windowHeight="15600" xr2:uid="{B01F5496-B8EA-4B4D-906B-0DA441535964}"/>
   </bookViews>
   <sheets>
     <sheet name="Test_1" sheetId="49" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>Water</t>
   </si>
@@ -54,6 +54,12 @@
   </si>
   <si>
     <t>Volumetric flow_m3/h</t>
+  </si>
+  <si>
+    <t>Propane</t>
+  </si>
+  <si>
+    <t>Carbon dioxide</t>
   </si>
 </sst>
 </file>
@@ -85,7 +91,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -121,11 +127,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -135,6 +150,9 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -485,8 +503,12 @@
       <c r="F1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4"/>
+      <c r="G1" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>7</v>
+      </c>
       <c r="I1" s="4"/>
       <c r="J1" s="4"/>
       <c r="K1" s="4"/>
@@ -533,10 +555,16 @@
         <v>4203.125</v>
       </c>
       <c r="E2">
-        <v>0.5</v>
+        <v>0.25</v>
       </c>
       <c r="F2">
-        <v>0.5</v>
+        <v>0.3</v>
+      </c>
+      <c r="G2">
+        <v>0.2</v>
+      </c>
+      <c r="H2">
+        <v>0.25</v>
       </c>
     </row>
     <row r="18" spans="17:17" x14ac:dyDescent="0.25">

</xml_diff>